<commit_message>
publish 2026-09-24 17:24 · 目录 v44
</commit_message>
<xml_diff>
--- a/模型价格目录大全.xlsx
+++ b/模型价格目录大全.xlsx
@@ -466,7 +466,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>生成 2026-09-24 10:21 ｜ 口径 USD/百万token（$/张、$/秒、$/次、$/小时单标）</t>
+          <t>生成 2026-09-24 17:24 ｜ 口径 USD/百万token（$/张、$/秒、$/次、$/小时单标）</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>枚举</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">

</xml_diff>